<commit_message>
Lições, Backlog, DER, Slide
</commit_message>
<xml_diff>
--- a/Sprint 2/Product Backlog + Matriz de Rastreabilidade dos Requisitos/Product Backlog - Safety Intelligence - Sprint 2.xlsx
+++ b/Sprint 2/Product Backlog + Matriz de Rastreabilidade dos Requisitos/Product Backlog - Safety Intelligence - Sprint 2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leona\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D15F9A1-51B1-41BF-870B-90BB3A17D064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{70694818-24EC-4269-8E65-A39C20383140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7F13FE21-3909-4024-9E51-F6B5B91CD81C}"/>
   </bookViews>
@@ -1090,6 +1090,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1117,9 +1120,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1127,629 +1127,11 @@
   <dxfs count="38">
     <dxf>
       <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border outline="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Tahoma"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFD24545"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1770,6 +1152,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1946,6 +1338,614 @@
         <name val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD24545"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Tahoma"/>
+        <family val="2"/>
+        <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -3123,45 +3123,45 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{18D1D61B-96A7-4717-8A7E-AB4616EE8DDA}" name="Tabela134" displayName="Tabela134" ref="A3:Q52" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" headerRowBorderDxfId="17" tableBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{18D1D61B-96A7-4717-8A7E-AB4616EE8DDA}" name="Tabela134" displayName="Tabela134" ref="A3:Q52" totalsRowShown="0" headerRowDxfId="37" dataDxfId="35" headerRowBorderDxfId="36" tableBorderDxfId="34">
   <autoFilter ref="A3:Q52" xr:uid="{2BF696E1-E460-4395-A8F6-CAA0467D7A56}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{08F9696B-A80C-4C31-8391-CAF183C1F64B}" name="Código do Requisito" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{6ED284F0-D736-42B0-9198-113881FC52C4}" name="Descrição do Requisito" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{86E74857-8436-47EC-8BEB-5963C142A460}" name="Tipo" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{3DCBA7DD-0B4C-4432-A78F-EA034FEBDBE5}" name="Importância" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{C3C6C53D-3038-436B-A369-C4378E80283E}" name="Status" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{CFFA1E83-FF4B-4BC4-B3C8-AA4FB1E5B750}" name="Tamanho" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{441C0D8E-35ED-4EF5-A300-48C37538B880}" name="Urgência" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{8EE8F4F1-94C0-4E2A-BAD0-4A78C47AECF9}" name="User Story" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{C08BB0DA-7C93-4314-BF50-531BDFEC181D}" name="Lean Ux Canvas" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{7B503E6B-0E6F-4AA8-A63B-9F05A061F43C}" name="Wireframe" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{678A4484-CA80-4328-A3AE-EE2479CDCB09}" name="Banco de Dados" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{E097E1F8-767A-420F-9B09-D2B473E00AE1}" name="Proto-Persona" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{38073914-2E9B-413C-99C9-687B22935A05}" name="Definição do Projeto" dataDxfId="4"/>
-    <tableColumn id="15" xr3:uid="{23D98D57-9ABF-4300-AAFB-6249D06E51DC}" name="Gestão" dataDxfId="3"/>
-    <tableColumn id="16" xr3:uid="{E2D244B6-F47E-40B5-8B5F-093ABCFAAB1F}" name="Website" dataDxfId="2"/>
-    <tableColumn id="17" xr3:uid="{A479396C-E100-4FF2-B848-EA0139317644}" name="Cloud" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{8B0CBAF9-476C-4CA2-A161-3B9DB0346272}" name="Custo" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{08F9696B-A80C-4C31-8391-CAF183C1F64B}" name="Código do Requisito" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{6ED284F0-D736-42B0-9198-113881FC52C4}" name="Descrição do Requisito" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{86E74857-8436-47EC-8BEB-5963C142A460}" name="Tipo" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{3DCBA7DD-0B4C-4432-A78F-EA034FEBDBE5}" name="Importância" dataDxfId="30"/>
+    <tableColumn id="9" xr3:uid="{C3C6C53D-3038-436B-A369-C4378E80283E}" name="Status" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{CFFA1E83-FF4B-4BC4-B3C8-AA4FB1E5B750}" name="Tamanho" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{441C0D8E-35ED-4EF5-A300-48C37538B880}" name="Urgência" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{8EE8F4F1-94C0-4E2A-BAD0-4A78C47AECF9}" name="User Story" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{C08BB0DA-7C93-4314-BF50-531BDFEC181D}" name="Lean Ux Canvas" dataDxfId="25"/>
+    <tableColumn id="11" xr3:uid="{7B503E6B-0E6F-4AA8-A63B-9F05A061F43C}" name="Wireframe" dataDxfId="24"/>
+    <tableColumn id="12" xr3:uid="{678A4484-CA80-4328-A3AE-EE2479CDCB09}" name="Banco de Dados" dataDxfId="23"/>
+    <tableColumn id="13" xr3:uid="{E097E1F8-767A-420F-9B09-D2B473E00AE1}" name="Proto-Persona" dataDxfId="22"/>
+    <tableColumn id="14" xr3:uid="{38073914-2E9B-413C-99C9-687B22935A05}" name="Definição do Projeto" dataDxfId="21"/>
+    <tableColumn id="15" xr3:uid="{23D98D57-9ABF-4300-AAFB-6249D06E51DC}" name="Gestão" dataDxfId="20"/>
+    <tableColumn id="16" xr3:uid="{E2D244B6-F47E-40B5-8B5F-093ABCFAAB1F}" name="Website" dataDxfId="19"/>
+    <tableColumn id="17" xr3:uid="{A479396C-E100-4FF2-B848-EA0139317644}" name="Cloud" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{8B0CBAF9-476C-4CA2-A161-3B9DB0346272}" name="Custo" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2BF696E1-E460-4395-A8F6-CAA0467D7A56}" name="Tabela1" displayName="Tabela1" ref="A2:H61" totalsRowShown="0" headerRowDxfId="37" dataDxfId="35" headerRowBorderDxfId="36" tableBorderDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2BF696E1-E460-4395-A8F6-CAA0467D7A56}" name="Tabela1" displayName="Tabela1" ref="A2:H61" totalsRowShown="0" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13">
   <autoFilter ref="A2:H61" xr:uid="{2BF696E1-E460-4395-A8F6-CAA0467D7A56}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{6ECC6F81-630B-49D3-805B-E9FE3D799D3D}" name="REQUISITO" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{1D058733-D303-4135-A124-29464DC33A73}" name="DESCRIÇÃO" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{4A9FBD53-C5AD-43F9-B80C-34C8759E680F}" name="CLASSIFICAÇÃO" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{6928EAB6-577B-4082-AAC3-4ABABECCFE53}" name="TAMANHO" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{CB0AD832-680E-4373-B96F-AFCC00E72603}" name="TAM(#)" dataDxfId="29">
+    <tableColumn id="1" xr3:uid="{6ECC6F81-630B-49D3-805B-E9FE3D799D3D}" name="REQUISITO" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{1D058733-D303-4135-A124-29464DC33A73}" name="DESCRIÇÃO" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{4A9FBD53-C5AD-43F9-B80C-34C8759E680F}" name="CLASSIFICAÇÃO" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{6928EAB6-577B-4082-AAC3-4ABABECCFE53}" name="TAMANHO" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{CB0AD832-680E-4373-B96F-AFCC00E72603}" name="TAM(#)" dataDxfId="8">
       <calculatedColumnFormula>IF(D3="P",5,IF(D3="PP",3,IF(D3="M",8,IF(D3="G",13,IF(D3="GG",21,"")))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{D7323832-7608-48DF-A6CD-B1E879E62D55}" name="PRIORIDADE" dataDxfId="28"/>
-    <tableColumn id="7" xr3:uid="{52683356-C07B-41EC-A6CD-AA16D06032D0}" name="SPRINT" dataDxfId="27"/>
-    <tableColumn id="8" xr3:uid="{77F999EF-0A37-433E-9457-E5928B79426C}" name="ESTADO" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{D7323832-7608-48DF-A6CD-B1E879E62D55}" name="PRIORIDADE" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{52683356-C07B-41EC-A6CD-AA16D06032D0}" name="SPRINT" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{77F999EF-0A37-433E-9457-E5928B79426C}" name="ESTADO" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3502,46 +3502,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="22"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="23"/>
     </row>
     <row r="2" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>103</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="24"/>
-      <c r="P2" s="24"/>
-      <c r="Q2" s="25"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="25"/>
+      <c r="P2" s="25"/>
+      <c r="Q2" s="26"/>
     </row>
     <row r="3" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -3574,13 +3574,13 @@
       <c r="J3" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="K3" s="29" t="s">
+      <c r="K3" s="20" t="s">
         <v>212</v>
       </c>
       <c r="L3" s="16" t="s">
         <v>213</v>
       </c>
-      <c r="M3" s="29" t="s">
+      <c r="M3" s="20" t="s">
         <v>214</v>
       </c>
       <c r="N3" s="16" t="s">
@@ -4034,7 +4034,7 @@
         <v>11</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F12" s="17">
         <v>8</v>
@@ -4140,7 +4140,7 @@
         <v>39</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F14" s="17">
         <v>8</v>
@@ -5412,7 +5412,7 @@
         <v>11</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F38" s="17">
         <v>21</v>
@@ -5465,7 +5465,7 @@
         <v>11</v>
       </c>
       <c r="E39" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F39" s="17">
         <v>21</v>
@@ -5518,7 +5518,7 @@
         <v>11</v>
       </c>
       <c r="E40" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F40" s="17">
         <v>21</v>
@@ -5571,7 +5571,7 @@
         <v>11</v>
       </c>
       <c r="E41" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F41" s="17">
         <v>21</v>
@@ -5624,7 +5624,7 @@
         <v>11</v>
       </c>
       <c r="E42" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F42" s="17">
         <v>21</v>
@@ -5730,7 +5730,7 @@
         <v>11</v>
       </c>
       <c r="E44" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F44" s="17">
         <v>21</v>
@@ -5836,7 +5836,7 @@
         <v>11</v>
       </c>
       <c r="E46" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F46" s="17">
         <v>8</v>
@@ -5889,7 +5889,7 @@
         <v>11</v>
       </c>
       <c r="E47" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F47" s="17">
         <v>13</v>
@@ -5942,7 +5942,7 @@
         <v>11</v>
       </c>
       <c r="E48" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F48" s="17">
         <v>21</v>
@@ -5995,7 +5995,7 @@
         <v>11</v>
       </c>
       <c r="E49" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F49" s="17">
         <v>13</v>
@@ -6048,7 +6048,7 @@
         <v>11</v>
       </c>
       <c r="E50" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F50" s="17">
         <v>8</v>
@@ -6101,7 +6101,7 @@
         <v>8</v>
       </c>
       <c r="E51" s="18" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
       <c r="F51" s="17">
         <v>21</v>
@@ -6165,13 +6165,13 @@
     <mergeCell ref="A2:Q2"/>
   </mergeCells>
   <conditionalFormatting sqref="E4:E52">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
       <formula>"Pronto"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
       <formula>"Planejado"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>"Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6214,16 +6214,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
@@ -7033,13 +7033,13 @@
       <c r="H31" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="K31" s="26" t="s">
+      <c r="K31" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="L31" s="26"/>
-      <c r="M31" s="26"/>
-      <c r="N31" s="26"/>
-      <c r="O31" s="26"/>
+      <c r="L31" s="27"/>
+      <c r="M31" s="27"/>
+      <c r="N31" s="27"/>
+      <c r="O31" s="27"/>
     </row>
     <row r="32" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
@@ -7808,10 +7808,10 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="H3:H61">
-    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"FINALIZADO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"PENDENTE"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8020,14 +8020,14 @@
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0432D9B1-72E5-4E34-937B-239DA2CDF102}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="48f4573d-ad3a-4e65-836d-04bb39ef68c7"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="48f4573d-ad3a-4e65-836d-04bb39ef68c7"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>

</xml_diff>